<commit_message>
Update model outputs 2026-06-15 18:30:57
</commit_message>
<xml_diff>
--- a/files/nznbl_upcoming.xlsx
+++ b/files/nznbl_upcoming.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t xml:space="preserve">Game Date</t>
   </si>
@@ -68,43 +68,52 @@
     <t xml:space="preserve">Q1 Total Ref</t>
   </si>
   <si>
-    <t xml:space="preserve">4 Jun</t>
+    <t xml:space="preserve">17 Jun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nelson Giants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manawatu Jets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PaceEff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 Jun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southland Sharks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taranaki Airs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19 Jun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canterbury Rams</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tauranga Whai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 Jun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auckland Tuatara</t>
   </si>
   <si>
     <t xml:space="preserve">Hawke s Bay Hawks</t>
   </si>
   <si>
-    <t xml:space="preserve">Nelson Giants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PaceEff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 Jun</t>
-  </si>
-  <si>
     <t xml:space="preserve">Otago Nuggets</t>
   </si>
   <si>
+    <t xml:space="preserve">21 Jun</t>
+  </si>
+  <si>
     <t xml:space="preserve">Franklin Bulls</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 Jun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Taranaki Airs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auckland Tuatara</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tauranga Whai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7 Jun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Southland Sharks</t>
   </si>
   <si>
     <t xml:space="preserve">Wellington Saints</t>
@@ -453,8 +462,8 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="11.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="19.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="18.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="18.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="19.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="12.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="12.71" hidden="0" customWidth="1"/>
@@ -542,46 +551,46 @@
         <v>21</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-0.26</v>
+        <v>-0.89</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>180.97</v>
+        <v>190.95</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-0.15</v>
+        <v>-0.17</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>-0.13</v>
+        <v>-0.45</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>90.48</v>
+        <v>95.47</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>-0.06</v>
+        <v>-0.22</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>45.24</v>
+        <v>47.74</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>-1.46</v>
+        <v>-1.12</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>182.57</v>
+        <v>180.59</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>-0.73</v>
+        <v>-0.56</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>91.29</v>
+        <v>90.3</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>-0.37</v>
+        <v>-0.28</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>45.64</v>
+        <v>45.15</v>
       </c>
     </row>
     <row r="3">
@@ -598,46 +607,46 @@
         <v>21</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-4.76</v>
+        <v>-18.43</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>192.91</v>
+        <v>173.91</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-0.15</v>
+        <v>-0.17</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>-2.38</v>
+        <v>-9.21</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>96.45</v>
+        <v>86.96</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>-1.19</v>
+        <v>-4.61</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>48.23</v>
+        <v>43.48</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>-4.86</v>
+        <v>-13.15</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>179.75</v>
+        <v>173.48</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>-2.43</v>
+        <v>-6.58</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>89.87</v>
+        <v>86.74</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>-1.21</v>
+        <v>-3.29</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>44.94</v>
+        <v>43.37</v>
       </c>
     </row>
     <row r="4">
@@ -654,110 +663,110 @@
         <v>21</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>18.74</v>
+        <v>-19.28</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>167.03</v>
+        <v>175.29</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>-0.15</v>
+        <v>-0.17</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>9.37</v>
+        <v>-9.64</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>83.51</v>
+        <v>87.65</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>4.69</v>
+        <v>-4.82</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>41.76</v>
+        <v>43.82</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>12.17</v>
+        <v>-12.73</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>175.3</v>
+        <v>179.91</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>6.09</v>
+        <v>-6.37</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>87.65</v>
+        <v>89.95</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>3.04</v>
+        <v>-3.18</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>43.82</v>
+        <v>44.98</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-1.43</v>
+        <v>-23.16</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>169.77</v>
+        <v>193.49</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>-0.15</v>
+        <v>-0.17</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-0.72</v>
+        <v>-11.58</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>84.88</v>
+        <v>96.74</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>-0.36</v>
+        <v>-5.79</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>42.44</v>
+        <v>48.37</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>-1.47</v>
+        <v>-14.3</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>179.93</v>
+        <v>183.7</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>-0.74</v>
+        <v>-7.15</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>89.96</v>
+        <v>91.85</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>-0.37</v>
+        <v>-3.58</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>44.98</v>
+        <v>45.93</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>24</v>
@@ -766,102 +775,102 @@
         <v>21</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-19.55</v>
+        <v>-3.36</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>207.42</v>
+        <v>165.28</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>-0.15</v>
+        <v>-0.17</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>-9.77</v>
+        <v>-1.68</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>103.71</v>
+        <v>82.64</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>-4.89</v>
+        <v>-0.84</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>51.85</v>
+        <v>41.32</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>-10.68</v>
+        <v>-5.2</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>190.18</v>
+        <v>166.97</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>-5.34</v>
+        <v>-2.6</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>95.09</v>
+        <v>83.48</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>-2.67</v>
+        <v>-1.3</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>47.55</v>
+        <v>41.74</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-15.22</v>
+        <v>12.56</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>173.61</v>
+        <v>184.24</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>-0.15</v>
+        <v>-0.17</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>-7.61</v>
+        <v>6.28</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>86.81</v>
+        <v>92.12</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>-3.81</v>
+        <v>3.14</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>43.4</v>
+        <v>46.06</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>-7.11</v>
+        <v>6.05</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>178.19</v>
+        <v>188.01</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>-3.56</v>
+        <v>3.03</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>89.1</v>
+        <v>94.01</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>-1.78</v>
+        <v>1.51</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>44.55</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-07-11 10:22:05
</commit_message>
<xml_diff>
--- a/files/nznbl_upcoming.xlsx
+++ b/files/nznbl_upcoming.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t xml:space="preserve">Game Date</t>
   </si>
@@ -68,55 +68,52 @@
     <t xml:space="preserve">Q1 Total Ref</t>
   </si>
   <si>
-    <t xml:space="preserve">20 Jun</t>
+    <t xml:space="preserve">11 Jul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manawatu Jets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hawke s Bay Hawks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PaceEff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southland Sharks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nelson Giants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 Jul</t>
   </si>
   <si>
     <t xml:space="preserve">Auckland Tuatara</t>
   </si>
   <si>
-    <t xml:space="preserve">Hawke s Bay Hawks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PaceEff</t>
-  </si>
-  <si>
     <t xml:space="preserve">Otago Nuggets</t>
   </si>
   <si>
+    <t xml:space="preserve">Wellington Saints</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canterbury Rams</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 Jul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 Jul</t>
+  </si>
+  <si>
     <t xml:space="preserve">Taranaki Airs</t>
   </si>
   <si>
-    <t xml:space="preserve">21 Jun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Franklin Bulls</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wellington Saints</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22 Jun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Southland Sharks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 Jun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tauranga Whai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25 Jun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manawatu Jets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26 Jun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nelson Giants</t>
+    <t xml:space="preserve">16 Jul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 Jul</t>
   </si>
 </sst>
 </file>
@@ -551,46 +548,46 @@
         <v>21</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-23.38</v>
+        <v>0.14</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>194.14</v>
+        <v>185.4</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-0.16</v>
+        <v>-0.13</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>-11.69</v>
+        <v>0.07</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>97.07</v>
+        <v>92.7</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>-5.85</v>
+        <v>0.04</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>48.54</v>
+        <v>46.35</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>-14.22</v>
+        <v>-2.58</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>183.72</v>
+        <v>184.93</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>-7.11</v>
+        <v>-1.29</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>91.86</v>
+        <v>92.46</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>-3.55</v>
+        <v>-0.65</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>45.93</v>
+        <v>46.23</v>
       </c>
     </row>
     <row r="3">
@@ -607,46 +604,46 @@
         <v>21</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-4.16</v>
+        <v>-8.88</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>166.34</v>
+        <v>184.28</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-0.16</v>
+        <v>-0.13</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>-2.08</v>
+        <v>-4.44</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>83.17</v>
+        <v>92.14</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>-1.04</v>
+        <v>-2.22</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>41.59</v>
+        <v>46.07</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>-5.32</v>
+        <v>-10.03</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>166.94</v>
+        <v>181.59</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>-2.66</v>
+        <v>-5.01</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>83.47</v>
+        <v>90.8</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>-1.33</v>
+        <v>-2.51</v>
       </c>
       <c r="R3" s="2" t="n">
-        <v>41.74</v>
+        <v>45.4</v>
       </c>
     </row>
     <row r="4">
@@ -663,54 +660,54 @@
         <v>21</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>12.04</v>
+        <v>-15.78</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>185.16</v>
+        <v>180.77</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>-0.16</v>
+        <v>-0.13</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>6.02</v>
+        <v>-7.89</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>92.58</v>
+        <v>90.38</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>3.01</v>
+        <v>-3.94</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>46.29</v>
+        <v>45.19</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>5.99</v>
+        <v>-11.65</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>187.94</v>
+        <v>177.19</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>2.99</v>
+        <v>-5.82</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>93.97</v>
+        <v>88.6</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>1.5</v>
+        <v>-2.91</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>46.99</v>
+        <v>44.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>20</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>28</v>
@@ -719,46 +716,46 @@
         <v>21</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>16.64</v>
+        <v>7.13</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>189.21</v>
+        <v>197.33</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>-0.16</v>
+        <v>-0.13</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>8.32</v>
+        <v>3.57</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>94.61</v>
+        <v>98.67</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>4.16</v>
+        <v>1.78</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>47.3</v>
+        <v>49.33</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>9.29</v>
+        <v>1.67</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>184.97</v>
+        <v>182.25</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>4.64</v>
+        <v>0.84</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>92.49</v>
+        <v>91.13</v>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>2.32</v>
+        <v>0.42</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>46.24</v>
+        <v>45.56</v>
       </c>
     </row>
     <row r="6">
@@ -766,167 +763,223 @@
         <v>29</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>13.95</v>
+        <v>7.72</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>169.69</v>
+        <v>184.31</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>-0.16</v>
+        <v>-0.13</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>6.97</v>
+        <v>3.86</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>84.84</v>
+        <v>92.15</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>3.49</v>
+        <v>1.93</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>42.42</v>
+        <v>46.08</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>8.83</v>
+        <v>0.01</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>177.85</v>
+        <v>179.32</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>4.42</v>
+        <v>0</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>88.92</v>
+        <v>89.66</v>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>2.21</v>
+        <v>0</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>44.46</v>
+        <v>44.83</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="C7" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1.38</v>
+        <v>0.1</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>178.09</v>
+        <v>171.72</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>-0.16</v>
+        <v>-0.13</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>0.69</v>
+        <v>0.05</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>89.05</v>
+        <v>85.86</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0.34</v>
+        <v>0.03</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>44.52</v>
+        <v>42.93</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0.93</v>
+        <v>-3.9</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>179.75</v>
+        <v>169.81</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>0.46</v>
+        <v>-1.95</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>89.88</v>
+        <v>84.9</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>0.23</v>
+        <v>-0.98</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>44.94</v>
+        <v>42.45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-16</v>
+        <v>-6.16</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>180.12</v>
+        <v>175.3</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>-0.16</v>
+        <v>-0.13</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>-8</v>
+        <v>-3.08</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>90.06</v>
+        <v>87.65</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>-4</v>
+        <v>-1.54</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>45.03</v>
+        <v>43.83</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>-10.65</v>
+        <v>-5.71</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>177.52</v>
+        <v>179.92</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>-5.32</v>
+        <v>-2.85</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>88.76</v>
+        <v>89.96</v>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>-2.66</v>
+        <v>-1.43</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>44.38</v>
+        <v>44.98</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>-23.32</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>190.91</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>-11.66</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>95.45</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>-5.83</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>47.73</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>-14.87</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>182.13</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>-7.44</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>91.06</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>-3.72</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>45.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>